<commit_message>
implemented "temporary file saving" process to reduce the likelihood of double-commits overwriting other workbooks.
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -640,10 +640,10 @@
         <v>On-site Support</v>
       </c>
       <c r="G2" t="str">
-        <v>Open</v>
+        <v>Closed</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>John</v>
       </c>
       <c r="I2" t="str">
         <v>2026-09-17</v>
@@ -652,13 +652,13 @@
         <v>14:09</v>
       </c>
       <c r="K2" t="str">
-        <v>Pending</v>
+        <v>Confirmed</v>
       </c>
       <c r="L2" t="str">
         <v>2026-09-17T02:34:25.526Z</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Resolved by test</v>
       </c>
       <c r="N2">
         <v>2.5</v>

</xml_diff>

<commit_message>
undid test read/writes to database, adjusted wording to have less customer-facing phrasing, modified on-site support appointment form to be able to support the 3 types of on-site support.
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -640,10 +640,10 @@
         <v>On-site Support</v>
       </c>
       <c r="G2" t="str">
-        <v>Closed</v>
+        <v>In Progress</v>
       </c>
       <c r="H2" t="str">
-        <v>John</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v>2026-09-17</v>
@@ -652,13 +652,13 @@
         <v>14:09</v>
       </c>
       <c r="K2" t="str">
-        <v>Confirmed</v>
+        <v>Pending</v>
       </c>
       <c r="L2" t="str">
         <v>2026-09-17T02:34:25.526Z</v>
       </c>
       <c r="M2" t="str">
-        <v>Resolved by test</v>
+        <v/>
       </c>
       <c r="N2">
         <v>2.5</v>

</xml_diff>

<commit_message>
Updated ticket details page to be more consistent. (displays technician instead of engineer + appointment status, but only when ticket is on-site support type.)
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -574,7 +574,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -746,9 +746,53 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>T-1789963309340</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>josiah wimbleton</v>
+      </c>
+      <c r="D5" t="str">
+        <v>ya@rawr.waow</v>
+      </c>
+      <c r="E5" t="str">
+        <v>hel</v>
+      </c>
+      <c r="F5" t="str">
+        <v>On-site Support</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Open</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-09-22</v>
+      </c>
+      <c r="J5" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L5" t="str">
+        <v>2026-09-21T04:01:49.340Z</v>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
adjusted on site (project) logic to be more accurate to requested specifications
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -714,7 +714,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -974,9 +974,56 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>T-1789984570988</v>
+      </c>
+      <c r="B7" t="str">
+        <v>C-0000000000004</v>
+      </c>
+      <c r="C7" t="str">
+        <v>josiah wimbleton</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ya@rawr.waow</v>
+      </c>
+      <c r="E7" t="str">
+        <v>helpppppppp</v>
+      </c>
+      <c r="F7" t="str">
+        <v>On-site Support</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Open</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>2026-09-30</v>
+      </c>
+      <c r="J7" t="str">
+        <v>03:00</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Pending</v>
+      </c>
+      <c r="L7" t="str">
+        <v>2026-09-21T09:56:10.988Z</v>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7">
+        <v>17</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Project</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>